<commit_message>
Clinical Sync - Published Ledger Inventory Base
</commit_message>
<xml_diff>
--- a/pearls_processed.xlsx
+++ b/pearls_processed.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,6 +478,446 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dennis-et-al-2026-recommendations-in-extracorporeal-cardiopulmonary-resuscitation-post-resuscitation-care-via-an.json</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-06-30 13:53:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1-s2.0-S2110582026001408-main.json</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:00:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>acc-003425.json</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:04:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>diagnostic_and_prognostic_value_of_the_venous.875.json</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>24</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:06:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>jcm-15-04227.json</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>31</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:07:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>jcm-15-04453.json</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:09:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PIIS2772930324000681.json</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>38</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:11:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PIIS2950133426001102.json</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>44</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:11:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>s10741-026-10636-0.json</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:15:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>s10877-026-01457-5.json</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>51</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:18:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>s40001-026-04401-0.json</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>58</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:19:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1-s2.0-S2772963X26002577-main.json</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>59</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:19:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>magnesium_sulfate_to_prevent_perioperative_atrial.847.json</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>62</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:20:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>s12245-025-01078-w.json</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:22:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>evidence_based,_cost_effective_management_of_lower.1388.json</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>71</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:25:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1-s2.0-S2667100X26000320-main.json</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>78</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:27:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>evidence_based,_cost_effective_management_of_upper.3.json</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:29:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>UEG Journal - 2026 - Cárdenas‐Jaén - AEG‐AESPANC‐OPGE‐SIED‐SPG Ibero‐Latin American Guidelines on Acute Pancreatitis .json</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>90</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:32:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PIIS103673142600041X.json</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>95</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:33:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>blood_bld-2023-022899-c-main.json</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>103</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:37:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1-s2.0-S1665268124005349-main.json</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>108</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026-06-30 14:37:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Chronic-hepatitis-B-in-2025--diagnosis--treatment-and-fut_2025_Clinical-Medi.json</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>117</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026-06-30 16:16:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>